<commit_message>
Correct phenotype thresholds and filter missing P values
Set the effective-marker calculation default to genome-wide significance (5e-8), report its adjusted threshold, and exclude missing P values during Step2 extraction. Use a fixed 1e-8 threshold for the five-summary example and clarify the workflow in the README.
</commit_message>
<xml_diff>
--- a/tools/run_metadata_template.xlsx
+++ b/tools/run_metadata_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\multipheno-gwas-viz\tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C0F2495-95C2-43DD-9B81-034F6D53D1C9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B55EC010-BCEB-45D2-8400-8AA420BAEF37}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="16650" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="16650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Study level" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="175">
   <si>
     <t>Field</t>
   </si>
@@ -211,12 +211,6 @@
   </si>
   <si>
     <t>Steps 5 and 7 - Catalog comparison</t>
-  </si>
-  <si>
-    <t>Step 5 matching window (bp)</t>
-  </si>
-  <si>
-    <t>Actual Step 5 window; Not applicable if skipped.</t>
   </si>
   <si>
     <t>Step 7 background window (bp)</t>
@@ -546,6 +540,30 @@
   </si>
   <si>
     <t>Agree, or have doubts</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Step 5 matching window (bp)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Actual Step 5 window; Not applicable if skipped.</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Actual delimiter used when constructing the map file. Default "; "</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>The delimiter used to separate Catalog labels in trait_2_catalog.csv</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>The reviewer of trait_2_catalog.csv</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Who carried out the review?</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -978,7 +996,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
@@ -1094,26 +1112,26 @@
     </row>
     <row r="13" spans="1:3" ht="29" customHeight="1">
       <c r="A13" s="12" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B13" s="13"/>
       <c r="C13" s="14"/>
     </row>
     <row r="14" spans="1:3" ht="48" customHeight="1">
       <c r="A14" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>165</v>
       </c>
       <c r="C14" s="10"/>
     </row>
     <row r="15" spans="1:3" ht="48" customHeight="1">
       <c r="A15" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>166</v>
       </c>
       <c r="C15" s="10"/>
     </row>
@@ -1327,21 +1345,39 @@
     </row>
     <row r="40" spans="1:3" ht="48" customHeight="1">
       <c r="A40" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="C40" s="10"/>
+    </row>
+    <row r="41" spans="1:3" ht="48" customHeight="1">
+      <c r="A41" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C41" s="10"/>
+    </row>
+    <row r="42" spans="1:3" ht="48" customHeight="1">
+      <c r="A42" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C42" s="10"/>
+    </row>
+    <row r="43" spans="1:3" ht="48" customHeight="1">
+      <c r="A43" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B43" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C40" s="10"/>
-    </row>
-    <row r="41" spans="1:3" ht="48" customHeight="1">
-      <c r="A41" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="B41" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="C41" s="11"/>
+      <c r="C43" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1384,24 +1420,24 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="31" customHeight="1">
       <c r="A2" s="15" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B2" s="16"/>
       <c r="C2" s="16"/>
@@ -1412,7 +1448,7 @@
     </row>
     <row r="3" spans="1:7" ht="29" customHeight="1">
       <c r="A3" s="12" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B3" s="13"/>
       <c r="C3" s="13"/>
@@ -1423,10 +1459,10 @@
     </row>
     <row r="4" spans="1:7" ht="48" customHeight="1">
       <c r="A4" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C4" s="8"/>
       <c r="D4" s="8"/>
@@ -1436,10 +1472,10 @@
     </row>
     <row r="5" spans="1:7" ht="48" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
@@ -1449,10 +1485,10 @@
     </row>
     <row r="6" spans="1:7" ht="48" customHeight="1">
       <c r="A6" s="5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
@@ -1462,10 +1498,10 @@
     </row>
     <row r="7" spans="1:7" ht="48" customHeight="1">
       <c r="A7" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
@@ -1475,10 +1511,10 @@
     </row>
     <row r="8" spans="1:7" ht="48" customHeight="1">
       <c r="A8" s="5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
@@ -1488,10 +1524,10 @@
     </row>
     <row r="9" spans="1:7" ht="48" customHeight="1">
       <c r="A9" s="5" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
@@ -1501,7 +1537,7 @@
     </row>
     <row r="10" spans="1:7" ht="29" customHeight="1">
       <c r="A10" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
@@ -1512,10 +1548,10 @@
     </row>
     <row r="11" spans="1:7" ht="48" customHeight="1">
       <c r="A11" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -1525,10 +1561,10 @@
     </row>
     <row r="12" spans="1:7" ht="48" customHeight="1">
       <c r="A12" s="5" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -1538,10 +1574,10 @@
     </row>
     <row r="13" spans="1:7" ht="48" customHeight="1">
       <c r="A13" s="5" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -1551,10 +1587,10 @@
     </row>
     <row r="14" spans="1:7" ht="48" customHeight="1">
       <c r="A14" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
@@ -1564,10 +1600,10 @@
     </row>
     <row r="15" spans="1:7" ht="48" customHeight="1">
       <c r="A15" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
@@ -1577,10 +1613,10 @@
     </row>
     <row r="16" spans="1:7" ht="48" customHeight="1">
       <c r="A16" s="5" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
@@ -1590,7 +1626,7 @@
     </row>
     <row r="17" spans="1:7" ht="29" customHeight="1">
       <c r="A17" s="12" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>
@@ -1601,10 +1637,10 @@
     </row>
     <row r="18" spans="1:7" ht="48" customHeight="1">
       <c r="A18" s="5" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
@@ -1614,10 +1650,10 @@
     </row>
     <row r="19" spans="1:7" ht="48" customHeight="1">
       <c r="A19" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
@@ -1627,7 +1663,7 @@
     </row>
     <row r="20" spans="1:7" ht="29" customHeight="1">
       <c r="A20" s="12" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
@@ -1638,10 +1674,10 @@
     </row>
     <row r="21" spans="1:7" ht="48" customHeight="1">
       <c r="A21" s="5" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
@@ -1651,10 +1687,10 @@
     </row>
     <row r="22" spans="1:7" ht="48" customHeight="1">
       <c r="A22" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
@@ -1664,10 +1700,10 @@
     </row>
     <row r="23" spans="1:7" ht="48" customHeight="1">
       <c r="A23" s="6" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="7"/>
@@ -1711,24 +1747,24 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>111</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="31" customHeight="1">
       <c r="A2" s="15" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B2" s="16"/>
       <c r="C2" s="16"/>
@@ -1739,7 +1775,7 @@
     </row>
     <row r="3" spans="1:7" ht="29" customHeight="1">
       <c r="A3" s="12" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B3" s="13"/>
       <c r="C3" s="13"/>
@@ -1750,10 +1786,10 @@
     </row>
     <row r="4" spans="1:7" ht="48" customHeight="1">
       <c r="A4" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -1763,10 +1799,10 @@
     </row>
     <row r="5" spans="1:7" ht="48" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -1776,7 +1812,7 @@
     </row>
     <row r="6" spans="1:7" ht="29" customHeight="1">
       <c r="A6" s="12" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B6" s="13"/>
       <c r="C6" s="13"/>
@@ -1787,10 +1823,10 @@
     </row>
     <row r="7" spans="1:7" ht="48" customHeight="1">
       <c r="A7" s="5" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -1800,10 +1836,10 @@
     </row>
     <row r="8" spans="1:7" ht="48" customHeight="1">
       <c r="A8" s="5" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -1813,10 +1849,10 @@
     </row>
     <row r="9" spans="1:7" ht="48" customHeight="1">
       <c r="A9" s="5" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -1826,10 +1862,10 @@
     </row>
     <row r="10" spans="1:7" ht="48" customHeight="1">
       <c r="A10" s="5" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -1839,10 +1875,10 @@
     </row>
     <row r="11" spans="1:7" ht="48" customHeight="1">
       <c r="A11" s="5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -1852,10 +1888,10 @@
     </row>
     <row r="12" spans="1:7" ht="48" customHeight="1">
       <c r="A12" s="5" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -1865,7 +1901,7 @@
     </row>
     <row r="13" spans="1:7" ht="29" customHeight="1">
       <c r="A13" s="12" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
@@ -1876,10 +1912,10 @@
     </row>
     <row r="14" spans="1:7" ht="48" customHeight="1">
       <c r="A14" s="5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
@@ -1889,10 +1925,10 @@
     </row>
     <row r="15" spans="1:7" ht="48" customHeight="1">
       <c r="A15" s="5" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
@@ -1902,10 +1938,10 @@
     </row>
     <row r="16" spans="1:7" ht="48" customHeight="1">
       <c r="A16" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
@@ -1915,10 +1951,10 @@
     </row>
     <row r="17" spans="1:7" ht="48" customHeight="1">
       <c r="A17" s="5" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
@@ -1928,10 +1964,10 @@
     </row>
     <row r="18" spans="1:7" ht="48" customHeight="1">
       <c r="A18" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
@@ -1941,7 +1977,7 @@
     </row>
     <row r="19" spans="1:7" ht="29" customHeight="1">
       <c r="A19" s="12" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
@@ -1952,10 +1988,10 @@
     </row>
     <row r="20" spans="1:7" ht="48" customHeight="1">
       <c r="A20" s="5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
@@ -1965,10 +2001,10 @@
     </row>
     <row r="21" spans="1:7" ht="48" customHeight="1">
       <c r="A21" s="5" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
@@ -1978,10 +2014,10 @@
     </row>
     <row r="22" spans="1:7" ht="48" customHeight="1">
       <c r="A22" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
@@ -1991,10 +2027,10 @@
     </row>
     <row r="23" spans="1:7" ht="48" customHeight="1">
       <c r="A23" s="5" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
@@ -2004,10 +2040,10 @@
     </row>
     <row r="24" spans="1:7" ht="48" customHeight="1">
       <c r="A24" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
@@ -2017,7 +2053,7 @@
     </row>
     <row r="25" spans="1:7" ht="29" customHeight="1">
       <c r="A25" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
@@ -2028,10 +2064,10 @@
     </row>
     <row r="26" spans="1:7" ht="48" customHeight="1">
       <c r="A26" s="5" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
@@ -2041,10 +2077,10 @@
     </row>
     <row r="27" spans="1:7" ht="48" customHeight="1">
       <c r="A27" s="5" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
@@ -2054,10 +2090,10 @@
     </row>
     <row r="28" spans="1:7" ht="48" customHeight="1">
       <c r="A28" s="5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
@@ -2067,10 +2103,10 @@
     </row>
     <row r="29" spans="1:7" ht="48" customHeight="1">
       <c r="A29" s="5" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
@@ -2080,10 +2116,10 @@
     </row>
     <row r="30" spans="1:7" ht="48" customHeight="1">
       <c r="A30" s="5" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
@@ -2093,10 +2129,10 @@
     </row>
     <row r="31" spans="1:7" ht="48" customHeight="1">
       <c r="A31" s="5" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
@@ -2106,10 +2142,10 @@
     </row>
     <row r="32" spans="1:7" ht="48" customHeight="1">
       <c r="A32" s="5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
@@ -2119,7 +2155,7 @@
     </row>
     <row r="33" spans="1:7" ht="29" customHeight="1">
       <c r="A33" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B33" s="13"/>
       <c r="C33" s="13"/>
@@ -2130,10 +2166,10 @@
     </row>
     <row r="34" spans="1:7" ht="48" customHeight="1">
       <c r="A34" s="5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
@@ -2143,10 +2179,10 @@
     </row>
     <row r="35" spans="1:7" ht="48" customHeight="1">
       <c r="A35" s="5" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
@@ -2156,10 +2192,10 @@
     </row>
     <row r="36" spans="1:7" ht="48" customHeight="1">
       <c r="A36" s="6" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C36" s="7"/>
       <c r="D36" s="7"/>

</xml_diff>